<commit_message>
site build 2026-10-08 21:18
</commit_message>
<xml_diff>
--- a/models/sovereigns/Nigeria_Sovereign_Model.xlsx
+++ b/models/sovereigns/Nigeria_Sovereign_Model.xlsx
@@ -652,7 +652,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CBN, 307th MPC Communiqué</t>
+          <t>CBN 307th MPC Communiqué</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -700,7 +700,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>NBS, Consumer Price Index Report August 2026</t>
+          <t>NBS Consumer Price Index Report August 2026</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -739,11 +739,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -778,12 +774,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Jun-26</t>
+          <t>30-Jun-26</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>DMO / IMF</t>
+          <t>DMO/IMF</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -793,7 +789,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>total public debt (federal, state and FCT; domestic and external) / GDP</t>
+          <t>Total public debt of ₦166.79T ($120.93B) at 30-Jun-26; the report labels the ratio both 'federal government' and 'total public', so the definition is unresolved</t>
         </is>
       </c>
     </row>
@@ -843,11 +839,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -882,12 +874,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2026 (stated as 'over 55%' of retained revenue; federal or consolidated basis unresolved)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>IMF Article IV / Budget Office</t>
+          <t>IMF Article IV concluding statement</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -895,11 +887,7 @@
           <t>01-Jun-26</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>federal interest payments as share of retained revenue; document states 'over 55%'</t>
-        </is>
-      </c>
+      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -947,11 +935,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1009,7 +993,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>CBN, Daily Foreign Exchange Reserves Bulletin</t>
+          <t>CBN Daily Foreign Exchange Reserves Bulletin</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1019,7 +1003,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>gross, CBN daily reserves bulletin (gold treatment not stated)</t>
+          <t>gross (CBN daily bulletin; the IMF monthly series incl. gold was 54.85 in Aug-26)</t>
         </is>
       </c>
     </row>
@@ -1056,12 +1040,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Oct-26</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Adjudicated document (gross reserves / imports of goods and services), IMF / CBN</t>
+          <t>IMF/CBN via prior adjudicated document (Medium)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1094,16 +1078,34 @@
           <t>external_debt_pct_gdp</t>
         </is>
       </c>
-      <c r="B20" s="2" t="n"/>
+      <c r="B20" s="2" t="n">
+        <v>14.4</v>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>% GDP</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>30-Jun-26</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>DMO Nigeria Public Debt Stock; IMF WEO</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>25-Sep-26</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>public external debt $54.52B (DMO, 30-Jun-26) divided by IMF WEO 2026E nominal GDP $377.4B; computed, public sector only</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1129,7 +1131,7 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>377.365</v>
+        <v>377.4</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1151,11 +1153,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1173,12 +1171,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Jun-26</t>
+          <t>30-Jun-26</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>DMO, Nigeria Public Debt Stock as at June 30, 2026</t>
+          <t>DMO Nigeria Public Debt Stock</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1374,8 +1372,14 @@
           <t>nominal_gdp_usd_bn</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" t="inlineStr"/>
+      <c r="B2" s="2" t="n">
+        <v>377.4</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>IMF WEO, 2026E</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1383,8 +1387,14 @@
           <t>real_gdp_growth_pct</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" t="inlineStr"/>
+      <c r="B3" s="2" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>IMF WEO, 2026E</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1401,8 +1411,14 @@
           <t>current_account_pct_gdp</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n"/>
-      <c r="C5" t="inlineStr"/>
+      <c r="B5" s="2" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>IMF WEO, 2026E</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1410,8 +1426,14 @@
           <t>fiscal_balance_pct_gdp</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" t="inlineStr"/>
+      <c r="B6" s="2" t="n">
+        <v>-4.4</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>IMF WEO, 2026E</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">

</xml_diff>

<commit_message>
site build 2026-10-16 14:37
</commit_message>
<xml_diff>
--- a/models/sovereigns/Nigeria_Sovereign_Model.xlsx
+++ b/models/sovereigns/Nigeria_Sovereign_Model.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>as of 09-Oct-26</t>
+          <t>as of 16-Oct-26</t>
         </is>
       </c>
     </row>
@@ -590,7 +590,7 @@
       <c r="D1" t="inlineStr"/>
       <c r="E1" t="inlineStr">
         <is>
-          <t>built 12-Oct-26 by pipeline/sovereign_model.py from database/sovereigns/nigeria.json</t>
+          <t>built 16-Oct-26 by pipeline/sovereign_model.py from database/sovereigns/nigeria.json</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>Apr-26</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -789,7 +789,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>DMO/IMF, Jun-26; label ambiguous between federal government and total public debt (total public debt ₦166.79T / $120.93B)</t>
+          <t>DMO total public debt / GDP; federal vs total public label unclear</t>
         </is>
       </c>
     </row>
@@ -836,7 +836,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>Apr-26</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -874,12 +874,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026, lower bound (&gt;55%), retained revenue; federal vs consolidated basis unresolved</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>IMF Article IV concluding statement</t>
+          <t>IMF Article IV concluding statement (lower bound, '&gt;55%' of federal retained revenue; basis unresolved)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -932,7 +932,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>Apr-26</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -979,7 +979,7 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>54.98</v>
+        <v>55.07</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -988,22 +988,22 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>05-Oct-26</t>
+          <t>09-Oct-26</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>CBN, Daily Foreign Exchange Reserves Bulletin</t>
+          <t>CBN via Nairametrics corrigendum</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>05-Oct-26</t>
+          <t>14-Oct-26</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>gross, CBN daily bulletin (IMF monthly series incl. gold: 54.85 in Aug-26; ex gold 51.78)</t>
+          <t>CBN headline gross, as corrected 14-Oct-26 (gold treatment not stated; IMF series incl. gold $54.85B Aug-26, ex gold $51.78B)</t>
         </is>
       </c>
     </row>
@@ -1038,19 +1038,15 @@
           <t>months</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Adjudicated prior document (IMF/CBN), Medium confidence</t>
+          <t>Adjudicated prior document (Medium confidence)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>16-Oct-26</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
@@ -1150,7 +1146,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>Apr-26</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -1321,7 +1317,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Aug-26</t>
+          <t>29-Aug-26</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1373,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>IMF WEO, 08-Oct-26</t>
+          <t>IMF WEO, Apr-26</t>
         </is>
       </c>
     </row>
@@ -1392,7 +1388,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>IMF WEO, 08-Oct-26</t>
+          <t>IMF WEO, Apr-26</t>
         </is>
       </c>
     </row>
@@ -1416,7 +1412,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>IMF WEO, 08-Oct-26</t>
+          <t>IMF WEO, Apr-26</t>
         </is>
       </c>
     </row>
@@ -1431,7 +1427,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>IMF WEO, 08-Oct-26</t>
+          <t>IMF WEO, Apr-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
site build 2026-10-26 10:04
</commit_message>
<xml_diff>
--- a/models/sovereigns/Nigeria_Sovereign_Model.xlsx
+++ b/models/sovereigns/Nigeria_Sovereign_Model.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>as of 16-Oct-26</t>
+          <t>as of 26-Oct-26</t>
         </is>
       </c>
     </row>
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>15.39</v>
+        <v>14.63</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -695,17 +695,17 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Aug-26</t>
+          <t>Sep-26</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>NBS, Consumer Price Index Report August 2026</t>
+          <t>NBS via Legit.ng, Tekedia, VON</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>15-Sep-26</t>
+          <t>15-Oct-26</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -736,7 +736,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Apr-26</t>
+          <t>13-Oct-26</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -774,12 +774,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Jun-26</t>
+          <t>30-Jun-26</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>DMO, Nigeria Public Debt Stock as at 30-Jun-26</t>
+          <t>DMO, Nigeria Public Debt Stock</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -789,7 +789,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>DMO total public debt / GDP; federal vs total public label unclear</t>
+          <t>total public debt (federal, states and FCT) per DMO; label unclear in source</t>
         </is>
       </c>
     </row>
@@ -836,7 +836,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Apr-26</t>
+          <t>13-Oct-26</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -865,7 +865,7 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>55</v>
+        <v>53.7</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -874,12 +874,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2026 (projection)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>IMF Article IV concluding statement (lower bound, '&gt;55%' of federal retained revenue; basis unresolved)</t>
+          <t>IMF Article IV via BusinessDay; federal or consolidated basis unresolved</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -913,7 +913,7 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>5.8</v>
+        <v>6.4</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -922,17 +922,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026E</t>
+          <t>2026F</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>IMF WEO</t>
+          <t>Fitch via Nairametrics</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Apr-26</t>
+          <t>10-Oct-26</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -1003,7 +1003,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>CBN headline gross, as corrected 14-Oct-26 (gold treatment not stated; IMF series incl. gold $54.85B Aug-26, ex gold $51.78B)</t>
+          <t>gross, CBN figure after downward revision from about 58 (corrigendum)</t>
         </is>
       </c>
     </row>
@@ -1031,22 +1031,26 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>9.199999999999999</v>
+        <v>6.3</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
           <t>months</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>end-2026F (months of current external payments, Fitch definition)</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Adjudicated prior document (Medium confidence)</t>
+          <t>Fitch via Nairametrics</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>16-Oct-26</t>
+          <t>10-Oct-26</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
@@ -1146,7 +1150,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Apr-26</t>
+          <t>13-Oct-26</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -1172,7 +1176,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>DMO, Nigeria Public Debt Stock as at 30-Jun-26</t>
+          <t>DMO, Nigeria Public Debt Stock (27.7% of external debt)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1268,12 +1272,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>10-Apr-26</t>
+          <t>09-Oct-26</t>
         </is>
       </c>
     </row>
@@ -1286,11 +1290,6 @@
       <c r="B30" t="inlineStr">
         <is>
           <t>B</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Stable</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1339,7 +1338,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1358,6 +1357,11 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>2027F</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Source</t>
         </is>
       </c>
@@ -1371,9 +1375,10 @@
       <c r="B2" s="2" t="n">
         <v>377.4</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>IMF WEO, Apr-26</t>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>IMF WEO, 13-Oct-26</t>
         </is>
       </c>
     </row>
@@ -1386,9 +1391,10 @@
       <c r="B3" s="2" t="n">
         <v>4.1</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>IMF WEO, Apr-26</t>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>IMF WEO, 13-Oct-26</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1405,8 @@
         </is>
       </c>
       <c r="B4" s="2" t="n"/>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1410,9 +1417,10 @@
       <c r="B5" s="2" t="n">
         <v>5.8</v>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>IMF WEO, Apr-26</t>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>IMF WEO, 13-Oct-26 (Fitch projects 6.4% for 2026)</t>
         </is>
       </c>
     </row>
@@ -1425,9 +1433,10 @@
       <c r="B6" s="2" t="n">
         <v>-4.4</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>IMF WEO, Apr-26</t>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>IMF WEO, 13-Oct-26</t>
         </is>
       </c>
     </row>
@@ -1438,7 +1447,8 @@
         </is>
       </c>
       <c r="B7" s="2" t="n"/>
-      <c r="C7" t="inlineStr"/>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1449,7 +1459,8 @@
       <c r="B8" s="2" t="n">
         <v>32.3</v>
       </c>
-      <c r="C8" t="inlineStr"/>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1458,7 +1469,8 @@
         </is>
       </c>
       <c r="B9" s="2" t="n"/>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1467,7 +1479,8 @@
         </is>
       </c>
       <c r="B10" s="2" t="n"/>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1476,7 +1489,8 @@
         </is>
       </c>
       <c r="B11" s="2" t="n"/>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1484,8 +1498,17 @@
           <t>interest_pct_revenue</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n"/>
-      <c r="C12" t="inlineStr"/>
+      <c r="B12" s="2" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>IMF Article IV via BusinessDay, 01-Jun-26</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>